<commit_message>
weekly update, 2022-03-02, SARS-CoV
</commit_message>
<xml_diff>
--- a/pdb/nsp3/SARS-CoV/domains_and_infos_of_nsp3.xlsx
+++ b/pdb/nsp3/SARS-CoV/domains_and_infos_of_nsp3.xlsx
@@ -7,16 +7,16 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="domain1" sheetId="1" r:id="rId1"/>
-    <sheet name="domain2" sheetId="2" r:id="rId2"/>
-    <sheet name="domain3" sheetId="3" r:id="rId3"/>
-    <sheet name="domain4" sheetId="4" r:id="rId4"/>
-    <sheet name="domain5" sheetId="5" r:id="rId5"/>
-    <sheet name="domain6" sheetId="6" r:id="rId6"/>
-    <sheet name="domain7" sheetId="7" r:id="rId7"/>
-    <sheet name="domain8" sheetId="8" r:id="rId8"/>
-    <sheet name="domain9" sheetId="9" r:id="rId9"/>
-    <sheet name="domain10" sheetId="10" r:id="rId10"/>
+    <sheet name="nsp3_Ubl1_" sheetId="1" r:id="rId1"/>
+    <sheet name="nsp3_Ubl2_nsp3_PL2pro_" sheetId="2" r:id="rId2"/>
+    <sheet name="nsp3_Ubl2_" sheetId="3" r:id="rId3"/>
+    <sheet name="nsp3_Macro3_" sheetId="4" r:id="rId4"/>
+    <sheet name="nsp3_PL2pro_" sheetId="5" r:id="rId5"/>
+    <sheet name="nsp3_NAB_" sheetId="6" r:id="rId6"/>
+    <sheet name="nsp3_Macro1_" sheetId="7" r:id="rId7"/>
+    <sheet name="nsp3_Macro2_" sheetId="8" r:id="rId8"/>
+    <sheet name="nsp3_DPUP_" sheetId="9" r:id="rId9"/>
+    <sheet name="multi-domain1" sheetId="10" r:id="rId10"/>
     <sheet name="Organisms" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="107">
   <si>
     <t>nsp3_Ubl1_</t>
   </si>
@@ -158,6 +158,15 @@
     <t>2008-08-23</t>
   </si>
   <si>
+    <t>7skq</t>
+  </si>
+  <si>
+    <t>BTSCOV-RF1.2004 PAPAIN-LIKE PROTEASE BOUND TO THE NON-COVALENT INHIBITOR GRL-0617</t>
+  </si>
+  <si>
+    <t>2021-10-21</t>
+  </si>
+  <si>
     <t>4ow0</t>
   </si>
   <si>
@@ -167,6 +176,12 @@
     <t>2014-01-28</t>
   </si>
   <si>
+    <t>7skr</t>
+  </si>
+  <si>
+    <t>BTSCOV-RF1.2004 PAPAIN-LIKE PROTEASE BOUND TO THE NON-COVALENT INHIBITOR 37</t>
+  </si>
+  <si>
     <t>nsp3_Macro3_</t>
   </si>
   <si>
@@ -318,6 +333,9 @@
   </si>
   <si>
     <t>homo sapiens</t>
+  </si>
+  <si>
+    <t>bat sars cov rf1/2004</t>
   </si>
   <si>
     <t>severe acute respiratory syndrome coronavirus</t>
@@ -739,7 +757,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -761,19 +779,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B3">
         <v>2.79</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -783,7 +801,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -791,12 +809,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -804,7 +822,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -822,22 +840,22 @@
     </row>
     <row r="6" spans="1:2">
       <c r="B6" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="B7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="B8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="B9" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -847,7 +865,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="B11" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -857,17 +875,17 @@
     </row>
     <row r="13" spans="1:2">
       <c r="B13" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="B14" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="B15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -877,12 +895,12 @@
     </row>
     <row r="17" spans="1:2">
       <c r="B17" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="B18" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -892,17 +910,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="B20" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="B21" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="B22" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -912,12 +930,12 @@
     </row>
     <row r="24" spans="1:2">
       <c r="B24" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
         <v>13</v>
@@ -925,7 +943,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s">
         <v>17</v>
@@ -948,7 +966,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
         <v>17</v>
@@ -956,7 +974,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="B34" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -976,25 +994,38 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
-        <v>99</v>
-      </c>
-      <c r="B41" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
-      <c r="A43" t="s">
-        <v>100</v>
-      </c>
-      <c r="B43" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="B40" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>104</v>
+      </c>
+      <c r="B42" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>106</v>
+      </c>
+      <c r="B46" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1195,7 +1226,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="110.7109375" customWidth="1"/>
@@ -1247,7 +1278,7 @@
         <v>44</v>
       </c>
       <c r="B4">
-        <v>2.1</v>
+        <v>3.16</v>
       </c>
       <c r="C4" t="s">
         <v>45</v>
@@ -1256,6 +1287,40 @@
         <v>15</v>
       </c>
       <c r="E4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5">
+        <v>2.1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6">
+        <v>2.89</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1276,7 +1341,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1298,87 +1363,87 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B7">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1398,7 +1463,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1420,19 +1485,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>2.5</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1452,7 +1517,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1474,19 +1539,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1506,7 +1571,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1528,36 +1593,36 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B3">
         <v>1.8</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B4">
         <v>1.4</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1577,7 +1642,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1599,36 +1664,36 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B3">
         <v>3.5</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B4">
         <v>2.22</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1648,7 +1713,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1670,36 +1735,36 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>